<commit_message>
Add to recycling and to refurbishment parameter files for JV2 script
</commit_message>
<xml_diff>
--- a/docs/Files/Tutorial6_JV_2/ODYM_T6_P5_ToUsedExportRate_V1.0.xlsx
+++ b/docs/Files/Tutorial6_JV_2/ODYM_T6_P5_ToUsedExportRate_V1.0.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E214718A-8B25-4594-BCA4-C143D7B944B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74EA42A7-193B-435C-AA08-145B078942AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="3" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="115">
   <si>
     <t>Format_Version</t>
   </si>
@@ -189,9 +189,6 @@
   </si>
   <si>
     <t>Steel shred</t>
-  </si>
-  <si>
-    <t>ODYM_Tutorial6_EoLRecoveryRate</t>
   </si>
   <si>
     <t>ODYM_Classifications_Master_Tutorial6_MaTrace</t>
@@ -821,7 +818,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>16</v>
@@ -835,7 +832,7 @@
         <v>18</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>16</v>
@@ -849,7 +846,7 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>16</v>
@@ -905,7 +902,7 @@
         <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>16</v>
@@ -919,7 +916,7 @@
         <v>24</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>16</v>
@@ -933,7 +930,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>16</v>
@@ -1003,7 +1000,7 @@
         <v>36</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>16</v>
@@ -1081,16 +1078,16 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>16</v>
@@ -1101,16 +1098,16 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" t="s">
         <v>72</v>
-      </c>
-      <c r="B24" t="s">
-        <v>73</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>16</v>
@@ -1121,16 +1118,16 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" t="s">
         <v>74</v>
-      </c>
-      <c r="B25" t="s">
-        <v>75</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>13</v>
       </c>
       <c r="D25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>16</v>
@@ -1141,10 +1138,10 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" t="s">
         <v>76</v>
-      </c>
-      <c r="B26" t="s">
-        <v>77</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>14</v>
@@ -1199,16 +1196,16 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>11</v>
@@ -1228,10 +1225,10 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
         <v>55</v>
@@ -1252,21 +1249,21 @@
         <v>54</v>
       </c>
       <c r="I2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="E3">
         <v>0.01</v>
@@ -1281,21 +1278,21 @@
         <v>54</v>
       </c>
       <c r="I3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="E4">
         <v>0.01</v>
@@ -1310,15 +1307,15 @@
         <v>54</v>
       </c>
       <c r="I4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C5" t="s">
         <v>55</v>
@@ -1339,15 +1336,15 @@
         <v>54</v>
       </c>
       <c r="I5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" t="s">
         <v>55</v>
@@ -1368,21 +1365,21 @@
         <v>54</v>
       </c>
       <c r="I6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="E7">
         <v>0.01</v>
@@ -1397,21 +1394,21 @@
         <v>54</v>
       </c>
       <c r="I7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="E8">
         <v>0.01</v>
@@ -1426,15 +1423,15 @@
         <v>54</v>
       </c>
       <c r="I8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C9" t="s">
         <v>55</v>
@@ -1455,7 +1452,7 @@
         <v>54</v>
       </c>
       <c r="I9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -1477,40 +1474,40 @@
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.3">
@@ -1522,13 +1519,13 @@
       </c>
       <c r="E3" s="15"/>
       <c r="F3" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H3" t="s">
         <v>90</v>
-      </c>
-      <c r="H3" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1543,52 +1540,52 @@
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="P2" s="2" t="s">
-        <v>105</v>
-      </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
-        <v>57</v>
+      <c r="B3" s="16" t="s">
+        <v>108</v>
       </c>
       <c r="C3">
         <v>1</v>

</xml_diff>